<commit_message>
Update software dataset (F-710-004-A Software.xlsx)
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/dataset/F-710-004-A Software.xlsx
+++ b/dataset/F-710-004-A Software.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SERG\Downloads\software-repository-main\software-repository-main\dataset\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76E5D9F5-F8FE-49CA-BD28-F720E8180442}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38E999B3-7EF8-4B64-B9FC-6E851DFFC3F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="6660" windowWidth="29040" windowHeight="15720" xr2:uid="{922D254A-B381-4E0E-8561-E0A75E953250}"/>
   </bookViews>
@@ -591,6 +591,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -609,7 +610,6 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -1189,10 +1189,10 @@
       <c r="G9" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="H9" s="31">
+      <c r="H9" s="32">
         <v>1500</v>
       </c>
-      <c r="I9" s="28" t="s">
+      <c r="I9" s="29" t="s">
         <v>60</v>
       </c>
     </row>
@@ -1218,8 +1218,8 @@
       <c r="G10" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="H10" s="32"/>
-      <c r="I10" s="29"/>
+      <c r="H10" s="33"/>
+      <c r="I10" s="30"/>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A11" s="15" t="s">
@@ -1243,8 +1243,8 @@
       <c r="G11" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="H11" s="33"/>
-      <c r="I11" s="30"/>
+      <c r="H11" s="34"/>
+      <c r="I11" s="31"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A12" s="15" t="s">
@@ -1435,10 +1435,10 @@
       <c r="B19" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="C19" s="34">
+      <c r="C19" s="28">
         <v>45910</v>
       </c>
-      <c r="D19" s="34">
+      <c r="D19" s="28">
         <v>46275</v>
       </c>
       <c r="E19" s="9" t="s">
@@ -1458,10 +1458,10 @@
       <c r="B20" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C20" s="34">
+      <c r="C20" s="28">
         <v>46052</v>
       </c>
-      <c r="D20" s="34">
+      <c r="D20" s="28">
         <v>46417</v>
       </c>
       <c r="E20" s="9" t="s">
@@ -1481,10 +1481,10 @@
       <c r="B21" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="C21" s="34">
+      <c r="C21" s="28">
         <v>46030</v>
       </c>
-      <c r="D21" s="34">
+      <c r="D21" s="28">
         <v>46395</v>
       </c>
       <c r="E21" s="9" t="s">
@@ -1504,10 +1504,10 @@
       <c r="B22" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="C22" s="34">
+      <c r="C22" s="28">
         <v>45935</v>
       </c>
-      <c r="D22" s="34">
+      <c r="D22" s="28">
         <v>46300</v>
       </c>
       <c r="E22" s="9" t="s">
@@ -1530,11 +1530,11 @@
       <c r="B23" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="C23" s="34">
+      <c r="C23" s="28">
         <v>46036</v>
       </c>
-      <c r="D23" s="34">
-        <v>46035</v>
+      <c r="D23" s="28">
+        <v>46400</v>
       </c>
       <c r="E23" s="9" t="s">
         <v>35</v>

</xml_diff>